<commit_message>
mudança para o acompanhamento de vendas de pre vencidos
</commit_message>
<xml_diff>
--- a/data/meta_supervisor.xlsx
+++ b/data/meta_supervisor.xlsx
@@ -2,21 +2,24 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
-  <workbookPr hidePivotFieldList="1" defaultThemeVersion="202300"/>
+  <workbookPr hidePivotFieldList="1"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\christian.roque\Desktop\Total_Day\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{97AB9520-F940-435A-A8CB-F69B50594BB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{14BCCA1B-8E86-46DC-B1B0-0E8813E79CDD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14016" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Planilha2" sheetId="4" r:id="rId1"/>
+    <sheet name="Planilha3" sheetId="6" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191028"/>
   <extLst>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+      <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
         <xcalcf:feature name="microsoft.com:RD"/>
@@ -36,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="26">
   <si>
     <t>FERNANDA DA SILVA OLIVEIRA</t>
   </si>
@@ -74,15 +77,9 @@
     <t>RILARY DIENIFER TRAUTMANN LIMA</t>
   </si>
   <si>
-    <t>WESLEY DE OLIVEIRA PAZ</t>
-  </si>
-  <si>
     <t>HERMANS SERGIO GUERREIRO SILVA - FARMA</t>
   </si>
   <si>
-    <t>LUIS REGINALDO ALMEIDA GOMES</t>
-  </si>
-  <si>
     <t>PAULO CESAR DAMACENA LEMOS - HB</t>
   </si>
   <si>
@@ -101,13 +98,25 @@
     <t>JONATHAS SANTOS ANDRADE - FARMA</t>
   </si>
   <si>
-    <t>BAIANA MEDICAMENTOS</t>
-  </si>
-  <si>
-    <t>nm_supervisor</t>
-  </si>
-  <si>
-    <t>meta_supervisor</t>
+    <t>META SUPERVISÃO</t>
+  </si>
+  <si>
+    <t>SUPERVISORES</t>
+  </si>
+  <si>
+    <t>MA</t>
+  </si>
+  <si>
+    <t>PI</t>
+  </si>
+  <si>
+    <t>NUBIA</t>
+  </si>
+  <si>
+    <t>cod_supervisor</t>
+  </si>
+  <si>
+    <t>cod_filial</t>
   </si>
 </sst>
 </file>
@@ -115,7 +124,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="_-[$R$-416]\ * #,##0.00_-;\-[$R$-416]\ * #,##0.00_-;_-[$R$-416]\ * &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="166" formatCode="_-[$R$-416]\ * #,##0.00_-;\-[$R$-416]\ * #,##0.00_-;_-[$R$-416]\ * &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
@@ -153,9 +162,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+  <cellXfs count="3">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -490,196 +502,308 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7656BC85-0027-461F-B9E3-11DEC5EEC80A}">
-  <dimension ref="A1:B23"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D95241F3-566F-482B-8E18-610590DC622A}">
+  <dimension ref="A1:D21"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="47.09765625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.19921875" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="8.796875" style="1"/>
+    <col min="2" max="2" width="13.19921875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="47.09765625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="18.09765625" style="2" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" s="1">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>125</v>
+      </c>
+      <c r="C2" t="s">
+        <v>1</v>
+      </c>
+      <c r="D2" s="2">
+        <v>56434.710574054472</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" s="1">
+        <v>1</v>
+      </c>
+      <c r="B3">
+        <v>106</v>
+      </c>
+      <c r="C3" t="s">
+        <v>3</v>
+      </c>
+      <c r="D3" s="2">
+        <v>22401.388181930193</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" s="1">
+        <v>1</v>
+      </c>
+      <c r="B4">
+        <v>145</v>
+      </c>
+      <c r="C4" t="s">
+        <v>4</v>
+      </c>
+      <c r="D4" s="2">
+        <v>24385.296244015291</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" s="1">
+        <v>3</v>
+      </c>
+      <c r="B5">
+        <v>43</v>
+      </c>
+      <c r="C5" t="s">
+        <v>0</v>
+      </c>
+      <c r="D5" s="2">
+        <v>9706.5791026598308</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" s="1">
+        <v>3</v>
+      </c>
+      <c r="B6">
+        <v>132</v>
+      </c>
+      <c r="C6" t="s">
+        <v>2</v>
+      </c>
+      <c r="D6" s="2">
+        <v>10263.581404307039</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" s="1">
+        <v>3</v>
+      </c>
+      <c r="B7">
+        <v>138</v>
+      </c>
+      <c r="C7" t="s">
+        <v>9</v>
+      </c>
+      <c r="D7" s="2">
+        <v>14706.442587246032</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" s="1">
+        <v>3</v>
+      </c>
+      <c r="B8">
+        <v>2</v>
+      </c>
+      <c r="C8" t="s">
+        <v>5</v>
+      </c>
+      <c r="D8" s="2">
+        <v>8468.1003918252809</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" s="1">
+        <v>3</v>
+      </c>
+      <c r="B9">
+        <v>46</v>
+      </c>
+      <c r="C9" t="s">
+        <v>6</v>
+      </c>
+      <c r="D9" s="2">
+        <v>12581.561513961791</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" s="1">
+        <v>7</v>
+      </c>
+      <c r="B10">
+        <v>95</v>
+      </c>
+      <c r="C10" t="s">
+        <v>12</v>
+      </c>
+      <c r="D10" s="2">
+        <v>33570.989999999991</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" s="1">
+        <v>7</v>
+      </c>
+      <c r="B11">
+        <v>50</v>
+      </c>
+      <c r="C11" t="s">
+        <v>18</v>
+      </c>
+      <c r="D11" s="2">
+        <v>33570.989999999991</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12" s="1">
+        <v>7</v>
+      </c>
+      <c r="B12">
+        <v>98</v>
+      </c>
+      <c r="C12" t="s">
+        <v>13</v>
+      </c>
+      <c r="D12" s="2">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A13" s="1">
+        <v>7</v>
+      </c>
+      <c r="B13">
+        <v>100</v>
+      </c>
+      <c r="C13" t="s">
+        <v>14</v>
+      </c>
+      <c r="D13" s="2">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A14" s="1">
+        <v>9</v>
+      </c>
+      <c r="B14">
+        <v>147</v>
+      </c>
+      <c r="C14" t="s">
+        <v>15</v>
+      </c>
+      <c r="D14" s="2">
+        <v>16062.948723594409</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A15" s="1">
+        <v>9</v>
+      </c>
+      <c r="B15">
+        <v>135</v>
+      </c>
+      <c r="C15" t="s">
+        <v>16</v>
+      </c>
+      <c r="D15" s="2">
+        <v>18277.770742394881</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A16" s="1">
+        <v>9</v>
+      </c>
+      <c r="B16">
+        <v>146</v>
+      </c>
+      <c r="C16" t="s">
+        <v>17</v>
+      </c>
+      <c r="D16" s="2">
+        <v>23357.445534010654</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A17" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B17">
+        <v>38</v>
+      </c>
+      <c r="C17" t="s">
+        <v>10</v>
+      </c>
+      <c r="D17" s="2">
+        <v>34511.134818759063</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A18" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B18">
+        <v>114</v>
+      </c>
+      <c r="C18" t="s">
+        <v>11</v>
+      </c>
+      <c r="D18" s="2">
+        <v>55042.375251074925</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A19" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B19">
+        <v>120</v>
+      </c>
+      <c r="C19" t="s">
+        <v>23</v>
+      </c>
+      <c r="D19" s="2">
+        <v>29334.464595945199</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A20" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" s="1">
-        <v>644202.57993250433</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" s="1">
-        <v>255711.98849212358</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>4</v>
-      </c>
-      <c r="B4" s="1">
-        <v>278358.31163162214</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>0</v>
-      </c>
-      <c r="B5" s="1">
-        <v>344193.33452228614</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>2</v>
-      </c>
-      <c r="B6" s="1">
-        <v>363944.52363977931</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>9</v>
-      </c>
-      <c r="B7" s="1">
-        <v>521487.48385285411</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>5</v>
-      </c>
-      <c r="B8" s="1">
-        <v>300277.12957422202</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>6</v>
-      </c>
-      <c r="B9" s="1">
-        <v>446139.63016085821</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>21</v>
-      </c>
-      <c r="B10" s="1">
-        <v>8215.4293970252875</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>13</v>
-      </c>
-      <c r="B11" s="1">
-        <v>185959.11317271218</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>20</v>
-      </c>
-      <c r="B12" s="1">
-        <v>197494.33805755054</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>14</v>
-      </c>
-      <c r="B13" s="1">
-        <v>7168.8570325169039</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>15</v>
-      </c>
-      <c r="B14" s="1">
-        <v>629007.95096420893</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>16</v>
-      </c>
-      <c r="B15" s="1">
-        <v>318561.63373848604</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>17</v>
-      </c>
-      <c r="B16" s="1">
-        <v>272251.89837604424</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>18</v>
-      </c>
-      <c r="B17" s="1">
-        <v>309791.05196232052</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>19</v>
-      </c>
-      <c r="B18" s="1">
-        <v>395886.77006163524</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>10</v>
-      </c>
-      <c r="B19" s="1">
-        <v>250152.17726092739</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>11</v>
-      </c>
-      <c r="B20" s="1">
-        <v>279806.36062682181</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>12</v>
-      </c>
-      <c r="B21" s="1">
-        <v>113878.31026225076</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
+      <c r="B20">
+        <v>69</v>
+      </c>
+      <c r="C20" t="s">
         <v>7</v>
       </c>
-      <c r="B22" s="1">
-        <v>478043.76420766662</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
+      <c r="D20" s="2">
+        <v>88809.584358607637</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A21" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B21">
+        <v>33</v>
+      </c>
+      <c r="C21" t="s">
         <v>8</v>
       </c>
-      <c r="B23" s="1">
-        <v>530236.07566108357</v>
+      <c r="D21" s="2">
+        <v>98505.720641392385</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
ajustando para o evento de vendas 9/9
</commit_message>
<xml_diff>
--- a/data/meta_supervisor.xlsx
+++ b/data/meta_supervisor.xlsx
@@ -2,24 +2,21 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
-  <workbookPr hidePivotFieldList="1"/>
+  <workbookPr hidePivotFieldList="1" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\christian.roque\Desktop\Total_Day\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{14BCCA1B-8E86-46DC-B1B0-0E8813E79CDD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{943C93E3-D57A-4BC5-ABA6-C04BD224D8F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14016" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="24240" windowHeight="13140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Planilha3" sheetId="6" r:id="rId1"/>
+    <sheet name="Planilha2" sheetId="3" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191028"/>
+  <calcPr calcId="191029"/>
   <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
         <xcalcf:feature name="microsoft.com:RD"/>
@@ -41,82 +38,82 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="26">
   <si>
+    <t>PI</t>
+  </si>
+  <si>
+    <t>MA</t>
+  </si>
+  <si>
+    <t>cod_filial</t>
+  </si>
+  <si>
+    <t>cod_supervisor</t>
+  </si>
+  <si>
+    <t>supervisores</t>
+  </si>
+  <si>
+    <t>meta supervisão</t>
+  </si>
+  <si>
+    <t>FERNANDO NOBRE MARTINS</t>
+  </si>
+  <si>
+    <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
+  </si>
+  <si>
+    <t>JOSE MARIA FERNANDES FONTENELE</t>
+  </si>
+  <si>
+    <t>MARIA ECILIA ALVES DOS SANTOS</t>
+  </si>
+  <si>
+    <t>VANILTON HOLANDA DA SILVA JUNIOR</t>
+  </si>
+  <si>
     <t>FERNANDA DA SILVA OLIVEIRA</t>
   </si>
   <si>
-    <t>FERNANDO NOBRE MARTINS</t>
-  </si>
-  <si>
     <t>JOSE FLAVIO DE SA AZEVEDO</t>
   </si>
   <si>
-    <t>JOSE MARIA FERNANDES FONTENELE</t>
-  </si>
-  <si>
-    <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
-  </si>
-  <si>
     <t>SALDANHA JUNIOR</t>
   </si>
   <si>
-    <t>VANILTON HOLANDA DA SILVA JUNIOR</t>
+    <t>PAULO CESAR DAMACENA LEMOS - HB</t>
+  </si>
+  <si>
+    <t>WELLINGTON NASCIMENTO SANTOS - HB</t>
+  </si>
+  <si>
+    <t>HERMANS SERGIO GUERREIRO SILVA - FARMA</t>
+  </si>
+  <si>
+    <t>JONATHAS SANTOS ANDRADE - FARMA</t>
+  </si>
+  <si>
+    <t>LOUIZE VANIELLE R. FARIAS (HNB RMR - PE)</t>
+  </si>
+  <si>
+    <t>JOSE CAETANO DA SILVA JUNIOR</t>
+  </si>
+  <si>
+    <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+  </si>
+  <si>
+    <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
   </si>
   <si>
     <t>EDEVANIA DA SILVA PEREIRA (PLUS)</t>
   </si>
   <si>
-    <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
-  </si>
-  <si>
-    <t>MARIA ECILIA ALVES DOS SANTOS</t>
-  </si>
-  <si>
     <t>BERNARDO TEIXEIRA COSTA NETO</t>
   </si>
   <si>
     <t>RILARY DIENIFER TRAUTMANN LIMA</t>
   </si>
   <si>
-    <t>HERMANS SERGIO GUERREIRO SILVA - FARMA</t>
-  </si>
-  <si>
-    <t>PAULO CESAR DAMACENA LEMOS - HB</t>
-  </si>
-  <si>
-    <t>WELLINGTON NASCIMENTO SANTOS - HB</t>
-  </si>
-  <si>
-    <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
-  </si>
-  <si>
-    <t>JOSE CAETANO DA SILVA JUNIOR</t>
-  </si>
-  <si>
-    <t>LOUIZE VANIELLE R. FARIAS (HNB RMR - PE)</t>
-  </si>
-  <si>
-    <t>JONATHAS SANTOS ANDRADE - FARMA</t>
-  </si>
-  <si>
-    <t>META SUPERVISÃO</t>
-  </si>
-  <si>
-    <t>SUPERVISORES</t>
-  </si>
-  <si>
-    <t>MA</t>
-  </si>
-  <si>
-    <t>PI</t>
-  </si>
-  <si>
-    <t>NUBIA</t>
-  </si>
-  <si>
-    <t>cod_supervisor</t>
-  </si>
-  <si>
-    <t>cod_filial</t>
+    <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
   </si>
 </sst>
 </file>
@@ -124,29 +121,21 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="166" formatCode="_-[$R$-416]\ * #,##0.00_-;\-[$R$-416]\ * #,##0.00_-;_-[$R$-416]\ * &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="165" formatCode="_-[$R$-416]\ * #,##0.00_-;\-[$R$-416]\ * #,##0.00_-;_-[$R$-416]\ * &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
-    <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Arial"/>
-    </font>
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="none"/>
     </fill>
   </fills>
   <borders count="1">
@@ -158,20 +147,15 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+  <cellXfs count="2">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 2" xfId="1" xr:uid="{679A0C32-DFAC-47A2-897B-49E0FD7E8CDE}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -502,308 +486,307 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D95241F3-566F-482B-8E18-610590DC622A}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A56F8248-F6E2-4ACE-AE7B-74CB24EA34E5}">
   <dimension ref="A1:D21"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="8.796875" style="1"/>
-    <col min="2" max="2" width="13.19921875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="47.09765625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="18.09765625" style="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="48.69921875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.5" style="1" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>25</v>
+      <c r="A1" t="s">
+        <v>2</v>
       </c>
       <c r="B1" t="s">
-        <v>24</v>
+        <v>3</v>
       </c>
       <c r="C1" t="s">
-        <v>20</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>19</v>
+        <v>4</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="1">
+      <c r="A2">
         <v>1</v>
       </c>
       <c r="B2">
         <v>125</v>
       </c>
       <c r="C2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D2" s="1">
+        <v>1269728.7716268308</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3">
         <v>1</v>
       </c>
-      <c r="D2" s="2">
-        <v>56434.710574054472</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="1">
+      <c r="B3">
+        <v>145</v>
+      </c>
+      <c r="C3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D3" s="1">
+        <v>545748.29481634218</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4">
         <v>1</v>
       </c>
-      <c r="B3">
+      <c r="B4">
         <v>106</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D4" s="1">
+        <v>530239.16272349597</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5">
         <v>3</v>
       </c>
-      <c r="D3" s="2">
-        <v>22401.388181930193</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" s="1">
-        <v>1</v>
-      </c>
-      <c r="B4">
-        <v>145</v>
-      </c>
-      <c r="C4" t="s">
-        <v>4</v>
-      </c>
-      <c r="D4" s="2">
-        <v>24385.296244015291</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" s="1">
+      <c r="B5">
+        <v>138</v>
+      </c>
+      <c r="C5" t="s">
+        <v>9</v>
+      </c>
+      <c r="D5" s="1">
+        <v>558770.79818590835</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6">
         <v>3</v>
       </c>
-      <c r="B5">
+      <c r="B6">
+        <v>46</v>
+      </c>
+      <c r="C6" t="s">
+        <v>10</v>
+      </c>
+      <c r="D6" s="1">
+        <v>453598.2330648721</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>3</v>
+      </c>
+      <c r="B7">
         <v>43</v>
       </c>
-      <c r="C5" t="s">
-        <v>0</v>
-      </c>
-      <c r="D5" s="2">
-        <v>9706.5791026598308</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" s="1">
+      <c r="C7" t="s">
+        <v>11</v>
+      </c>
+      <c r="D7" s="1">
+        <v>401184.36881949956</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8">
         <v>3</v>
       </c>
-      <c r="B6">
+      <c r="B8">
         <v>132</v>
       </c>
-      <c r="C6" t="s">
+      <c r="C8" t="s">
+        <v>12</v>
+      </c>
+      <c r="D8" s="1">
+        <v>379527.96466602071</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>3</v>
+      </c>
+      <c r="B9">
         <v>2</v>
       </c>
-      <c r="D6" s="2">
-        <v>10263.581404307039</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" s="1">
-        <v>3</v>
-      </c>
-      <c r="B7">
-        <v>138</v>
-      </c>
-      <c r="C7" t="s">
+      <c r="C9" t="s">
+        <v>13</v>
+      </c>
+      <c r="D9" s="1">
+        <v>302203.85443036543</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>7</v>
+      </c>
+      <c r="B10">
+        <v>98</v>
+      </c>
+      <c r="C10" t="s">
+        <v>14</v>
+      </c>
+      <c r="D10" s="1">
+        <v>806098.12525992142</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>7</v>
+      </c>
+      <c r="B11">
+        <v>100</v>
+      </c>
+      <c r="C11" t="s">
+        <v>15</v>
+      </c>
+      <c r="D11" s="1">
+        <v>425730.7363007958</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>7</v>
+      </c>
+      <c r="B12">
+        <v>95</v>
+      </c>
+      <c r="C12" t="s">
+        <v>16</v>
+      </c>
+      <c r="D12" s="1">
+        <v>230789.9599278653</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <v>7</v>
+      </c>
+      <c r="B13">
+        <v>50</v>
+      </c>
+      <c r="C13" t="s">
+        <v>17</v>
+      </c>
+      <c r="D13" s="1">
+        <v>194216.32184475061</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A14">
         <v>9</v>
       </c>
-      <c r="D7" s="2">
-        <v>14706.442587246032</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8" s="1">
-        <v>3</v>
-      </c>
-      <c r="B8">
-        <v>2</v>
-      </c>
-      <c r="C8" t="s">
-        <v>5</v>
-      </c>
-      <c r="D8" s="2">
-        <v>8468.1003918252809</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" s="1">
-        <v>3</v>
-      </c>
-      <c r="B9">
-        <v>46</v>
-      </c>
-      <c r="C9" t="s">
-        <v>6</v>
-      </c>
-      <c r="D9" s="2">
-        <v>12581.561513961791</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10" s="1">
-        <v>7</v>
-      </c>
-      <c r="B10">
-        <v>95</v>
-      </c>
-      <c r="C10" t="s">
-        <v>12</v>
-      </c>
-      <c r="D10" s="2">
-        <v>33570.989999999991</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11" s="1">
-        <v>7</v>
-      </c>
-      <c r="B11">
-        <v>50</v>
-      </c>
-      <c r="C11" t="s">
+      <c r="B14">
+        <v>146</v>
+      </c>
+      <c r="C14" t="s">
         <v>18</v>
       </c>
-      <c r="D11" s="2">
-        <v>33570.989999999991</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12" s="1">
-        <v>7</v>
-      </c>
-      <c r="B12">
-        <v>98</v>
-      </c>
-      <c r="C12" t="s">
-        <v>13</v>
-      </c>
-      <c r="D12" s="2">
-        <v>15000</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A13" s="1">
-        <v>7</v>
-      </c>
-      <c r="B13">
-        <v>100</v>
-      </c>
-      <c r="C13" t="s">
-        <v>14</v>
-      </c>
-      <c r="D13" s="2">
-        <v>15000</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A14" s="1">
-        <v>9</v>
-      </c>
-      <c r="B14">
-        <v>147</v>
-      </c>
-      <c r="C14" t="s">
-        <v>15</v>
-      </c>
-      <c r="D14" s="2">
-        <v>16062.948723594409</v>
+      <c r="D14" s="1">
+        <v>429705.98547714611</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A15" s="1">
+      <c r="A15">
         <v>9</v>
       </c>
       <c r="B15">
         <v>135</v>
       </c>
       <c r="C15" t="s">
-        <v>16</v>
-      </c>
-      <c r="D15" s="2">
-        <v>18277.770742394881</v>
+        <v>19</v>
+      </c>
+      <c r="D15" s="1">
+        <v>374775.32536699361</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A16" s="1">
+      <c r="A16">
         <v>9</v>
       </c>
       <c r="B16">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="C16" t="s">
-        <v>17</v>
-      </c>
-      <c r="D16" s="2">
-        <v>23357.445534010654</v>
+        <v>20</v>
+      </c>
+      <c r="D16" s="1">
+        <v>364830.59568110958</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A17" s="1" t="s">
+      <c r="A17" t="s">
+        <v>0</v>
+      </c>
+      <c r="B17">
+        <v>39</v>
+      </c>
+      <c r="C17" t="s">
         <v>21</v>
       </c>
-      <c r="B17">
+      <c r="D17" s="1">
+        <v>967286.30113893328</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>0</v>
+      </c>
+      <c r="B18">
+        <v>69</v>
+      </c>
+      <c r="C18" t="s">
+        <v>22</v>
+      </c>
+      <c r="D18" s="1">
+        <v>691106.01136106486</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>1</v>
+      </c>
+      <c r="B19">
         <v>38</v>
-      </c>
-      <c r="C17" t="s">
-        <v>10</v>
-      </c>
-      <c r="D17" s="2">
-        <v>34511.134818759063</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A18" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="B18">
-        <v>114</v>
-      </c>
-      <c r="C18" t="s">
-        <v>11</v>
-      </c>
-      <c r="D18" s="2">
-        <v>55042.375251074925</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A19" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="B19">
-        <v>120</v>
       </c>
       <c r="C19" t="s">
         <v>23</v>
       </c>
-      <c r="D19" s="2">
-        <v>29334.464595945199</v>
+      <c r="D19" s="1">
+        <v>645011.17730252154</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A20" s="1" t="s">
-        <v>22</v>
+      <c r="A20" t="s">
+        <v>1</v>
       </c>
       <c r="B20">
-        <v>69</v>
+        <v>114</v>
       </c>
       <c r="C20" t="s">
-        <v>7</v>
-      </c>
-      <c r="D20" s="2">
-        <v>88809.584358607637</v>
+        <v>24</v>
+      </c>
+      <c r="D20" s="1">
+        <v>519393.11883568548</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A21" s="1" t="s">
-        <v>22</v>
+      <c r="A21" t="s">
+        <v>1</v>
       </c>
       <c r="B21">
-        <v>33</v>
+        <v>120</v>
       </c>
       <c r="C21" t="s">
-        <v>8</v>
-      </c>
-      <c r="D21" s="2">
-        <v>98505.720641392385</v>
+        <v>25</v>
+      </c>
+      <c r="D21" s="1">
+        <v>474510.38562012545</v>
       </c>
     </row>
   </sheetData>

</xml_diff>